<commit_message>
refactored user authentication into separate router and updated project configuration
</commit_message>
<xml_diff>
--- a/Oceano.xlsx
+++ b/Oceano.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/swarnjeetsingh/Documents/Projects/ecomm-oceano/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05AB04DB-4314-EA41-AD7E-BB7BA3E9265E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0776343F-6AB2-2B4F-8411-5A760119A269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{446970C8-80E2-C142-9FB9-D5D8363202F8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -128,9 +128,6 @@
     <t>varchar(100)</t>
   </si>
   <si>
-    <t>varchar(254)</t>
-  </si>
-  <si>
     <t>varchar(50)</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>auto increment</t>
   </si>
   <si>
-    <t>default</t>
-  </si>
-  <si>
     <t>enum userType { "ADMIN", "DISTRIBUTOR", "CONSUMER"}</t>
   </si>
   <si>
@@ -162,6 +156,18 @@
   </si>
   <si>
     <t>modifiedBy</t>
+  </si>
+  <si>
+    <t>varchar(60)</t>
+  </si>
+  <si>
+    <t>default value</t>
+  </si>
+  <si>
+    <t>role</t>
+  </si>
+  <si>
+    <t>long</t>
   </si>
 </sst>
 </file>
@@ -561,191 +567,166 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEFC89BF-E8B0-C940-89D4-DE60F3EC282B}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.1640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.1640625" style="1"/>
-    <col min="2" max="2" width="18.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1640625" style="1"/>
-    <col min="6" max="6" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="1"/>
-    <col min="8" max="8" width="14.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.1640625" style="1"/>
-    <col min="10" max="10" width="15.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="35" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="13.1640625" style="1"/>
+    <col min="1" max="1" width="18.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" style="1"/>
+    <col min="5" max="5" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" style="1"/>
+    <col min="7" max="7" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="1"/>
+    <col min="9" max="9" width="15.6640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="35" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="13.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="1">
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1">
+        <v>9891796895</v>
+      </c>
+      <c r="H2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="I2" s="1">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="1">
-        <v>9891796895</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1</v>
-      </c>
-      <c r="J2" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="3"/>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="1" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="3"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="1" t="s">
+    </row>
+    <row r="8" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1</v>
+      </c>
+      <c r="I8" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8" s="1">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{CF741AA7-E5B0-8E4D-9AC5-33B6DCBAE721}"/>
-    <hyperlink ref="D2" r:id="rId2" xr:uid="{F4AB8F9F-A9C1-2148-BD63-858F07F5B7B1}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{CF741AA7-E5B0-8E4D-9AC5-33B6DCBAE721}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{F4AB8F9F-A9C1-2148-BD63-858F07F5B7B1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -802,16 +783,16 @@
         <v>12</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>